<commit_message>
Add condition of min controllable capacity as new scenario
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_min_controllable_capacity.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_min_controllable_capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0E8A32A-0C6F-4938-9321-9ADC428A92D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAD0FB5-1947-4DD4-BB47-B43D68D91140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,13 +56,13 @@
     <t>Attribute</t>
   </si>
   <si>
-    <t>NCAP_BND</t>
-  </si>
-  <si>
     <t>LimType</t>
   </si>
   <si>
     <t>LO</t>
+  </si>
+  <si>
+    <t>CAP_BND</t>
   </si>
 </sst>
 </file>
@@ -403,7 +403,7 @@
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4">
         <v>2030</v>
@@ -426,10 +426,10 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5">
         <v>2</v>

</xml_diff>

<commit_message>
Adding battery storage to UC_min_solid_2035
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_min_controllable_capacity.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_min_controllable_capacity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEB3C8E-AE26-439E-B463-68EA6E0E99DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F3835F-325C-4E53-9E8E-0F4A3BE5DA1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,10 +77,10 @@
     <t>UC_min_solid_2035</t>
   </si>
   <si>
-    <t>pp_controllable</t>
-  </si>
-  <si>
     <t>Minimum solid fuel power plants penetration</t>
+  </si>
+  <si>
+    <t>pp_controllable,Util Batt Stg</t>
   </si>
 </sst>
 </file>
@@ -408,8 +408,8 @@
   <dimension ref="B3:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
@@ -456,7 +456,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>2030</v>
@@ -471,12 +471,12 @@
         <v>2</v>
       </c>
       <c r="J7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8">
         <v>2035</v>
@@ -493,7 +493,7 @@
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>0</v>

</xml_diff>